<commit_message>
feat: Enhance workbook product handling in storefront
- Introduced live product management in category and product detail pages.
- Added deduplication and selection logic for live products based on workbook entries.
- Created a new utility module for handling live product lookups and category candidates.
- Updated category page to display live product stock and details.
- Improved product detail page to resolve workbook product IDs and ensure stock actions are enabled.
- Added CSS styles for product stock display.
- Implemented tests for category and product detail pages to validate new functionality.
- Ensured storefront schema is repaired during catalog import to maintain data integrity.
</commit_message>
<xml_diff>
--- a/artifacts/import-templates/catalog-import-sample-workbook.xlsx
+++ b/artifacts/import-templates/catalog-import-sample-workbook.xlsx
@@ -299,7 +299,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -358,7 +358,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>men</t>
+          <t>mens</t>
         </is>
       </c>
     </row>
@@ -370,19 +370,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>mens</t>
+          <t>nam</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>shop-men</t>
+          <t>atelier-women</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>nam</t>
+          <t>Shop Women</t>
         </is>
       </c>
     </row>
@@ -394,7 +394,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Shop Women</t>
+          <t>shop-women</t>
         </is>
       </c>
     </row>
@@ -406,7 +406,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>shop-women</t>
+          <t>Women</t>
         </is>
       </c>
     </row>
@@ -418,7 +418,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>nu</t>
         </is>
       </c>
     </row>
@@ -430,31 +430,31 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>women</t>
+          <t>atelier-women</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>atelier-women</t>
+          <t>footwear</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>nu</t>
+          <t>Footwear</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>atelier-women</t>
+          <t>footwear</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>atelier-women</t>
+          <t>shoes</t>
         </is>
       </c>
     </row>
@@ -466,7 +466,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>giay</t>
         </is>
       </c>
     </row>
@@ -478,43 +478,43 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>footwear</t>
+          <t>footwear-atelier</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>footwear</t>
+          <t>accessories</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>shoes</t>
+          <t>Accessories</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>footwear</t>
+          <t>accessories</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>giay</t>
+          <t>accessory</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>footwear</t>
+          <t>accessories</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>footwear-atelier</t>
+          <t>phu kien</t>
         </is>
       </c>
     </row>
@@ -525,54 +525,6 @@
         </is>
       </c>
       <c r="B19" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>accessories</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>accessories</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>accessories</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>accessory</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>accessories</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>phu kien</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>accessories</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
         <is>
           <t>accessories-atelier</t>
         </is>

</xml_diff>